<commit_message>
feat: add role-based policy engine and C-drive protection
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -540,7 +540,6 @@
           <t>Plan composite + ask confirm + execute 3 steps</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -551,9 +550,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -566,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -676,7 +672,6 @@
           <t>Denied by policy</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -687,9 +682,180 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Delete file in C</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Role=user, path=C:/tmp/a.txt</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>xoa file C:/tmp/a.txt</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Denied by policy</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Flow 01 rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Delete file in C</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Role=owner, allow_c_drive_full=false</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>xoa file C:/tmp/a.txt</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Denied unless owner enables full C drive</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Flow 01 rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Delete file in C</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Role=dev, DEV_SECRET valid</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>xoa file C:/tmp/a.txt</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Allowed</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Flow 01 rule</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -702,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -812,7 +978,6 @@
           <t>Must require explicit confirm</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -823,9 +988,64 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Policy audit logging</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Any executable command</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>run command</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Policy checks written to data/audit.jsonl</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Flow 01 log control</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -948,7 +1168,6 @@
           <t>Session unlock for next command</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -959,9 +1178,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -974,7 +1190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1084,7 +1300,6 @@
           <t>find_draft action generated</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -1095,9 +1310,64 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Composite policy flatten</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Composite action includes mixed risk</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>find + zalo + bulk email</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Each sub-action evaluated by policy</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Flow 01 core behavior</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: enforce session-bound execution and identity hardening
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,130 @@
       <c r="I2" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Session required run</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>No active session</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>python run.py run "tim file o d"</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Command denied with login prompt</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Flow 02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>F-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Login and run</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Valid login</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>login then run</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Run executes with session-bound user context</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Flow 02</t>
         </is>
       </c>
     </row>
@@ -714,7 +838,6 @@
           <t>Denied by policy</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -772,7 +895,6 @@
           <t>Denied unless owner enables full C drive</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -830,7 +952,6 @@
           <t>Allowed</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -863,6 +984,311 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>High-risk outbound</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bulk recipients &gt; 5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>gui email hang loat</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Must require explicit confirm</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Policy audit logging</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Any executable command</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>run command</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Policy checks written to data/audit.jsonl</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Flow 01 log control</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Auth lockout</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Repeated wrong PIN/secret</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>multiple failed logins</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Actor locked for AUTH_LOCK_MINUTES</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Flow 02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sensitive rate limit</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>session active</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>many sensitive actions quickly</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Rate limit denial after threshold</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Flow 02</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -950,32 +1376,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S-001</t>
+          <t>V-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>High-risk outbound</t>
+          <t>Wakeword VN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>owner</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bulk recipients &gt; 5</t>
+          <t>Mic active</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>gui email hang loat</t>
+          <t>noi wakeword</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Must require explicit confirm</t>
+          <t>Session unlock for next command</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -985,19 +1411,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S-002</t>
+          <t>V-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Policy audit logging</t>
+          <t>Voice confidence fallback</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1007,17 +1433,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Any executable command</t>
+          <t>confidence below threshold</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>run command</t>
+          <t>login with low confidence + PIN</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Policy checks written to data/audit.jsonl</t>
+          <t>Authentication succeeds only with valid PIN</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -1043,7 +1469,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Flow 01 log control</t>
+          <t>Flow 02</t>
         </is>
       </c>
     </row>
@@ -1052,13 +1478,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1140,138 +1566,6 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>V-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Wakeword VN</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Mic active</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>noi wakeword</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Session unlock for next command</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Flow</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Precondition</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Actual</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
           <t>R-001</t>
         </is>
       </c>
@@ -1342,7 +1636,6 @@
           <t>Each sub-action evaluated by policy</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -1366,6 +1659,68 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>Flow 01 core behavior</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Session revoke</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Active session exists</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>logout then run</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Run denied until login again</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Flow 02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: upgrade vietnamese voice flow and automate testcase execution
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -540,14 +540,29 @@
           <t>Plan composite + ask confirm + execute 3 steps</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>steps=3</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Composite run as owner.</t>
         </is>
       </c>
     </row>
@@ -796,14 +811,29 @@
           <t>Denied by policy</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Guest cannot modify files.</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>Critical</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Guest delete C must deny.</t>
         </is>
       </c>
     </row>
@@ -838,9 +868,14 @@
           <t>Denied by policy</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>User cannot delete on C drive.</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -860,7 +895,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Flow 01 rule</t>
+          <t>User delete C must deny.</t>
         </is>
       </c>
     </row>
@@ -895,9 +930,14 @@
           <t>Denied unless owner enables full C drive</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Owner must enable full C access to delete in C drive.</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -917,7 +957,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Flow 01 rule</t>
+          <t>Owner without toggle must deny.</t>
         </is>
       </c>
     </row>
@@ -952,9 +992,14 @@
           <t>Allowed</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Dev full access on C drive.</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -974,7 +1019,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Flow 01 rule</t>
+          <t>Dev delete C allowed.</t>
         </is>
       </c>
     </row>
@@ -1099,14 +1144,29 @@
           <t>Must require explicit confirm</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>allowed=True, confirm=True</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>Critical</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>High-risk outbound confirmation.</t>
         </is>
       </c>
     </row>
@@ -1141,9 +1201,14 @@
           <t>Policy checks written to data/audit.jsonl</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>audit_exists=True</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1163,7 +1228,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Flow 01 log control</t>
+          <t>Audit log exists.</t>
         </is>
       </c>
     </row>
@@ -1198,10 +1263,14 @@
           <t>Actor locked for AUTH_LOCK_MINUTES</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Actor is locked until 2026-03-21T16:52:03.993437+00:00.</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1221,7 +1290,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Flow 02</t>
+          <t>Actor lockout after repeated failures.</t>
         </is>
       </c>
     </row>
@@ -1256,10 +1325,14 @@
           <t>Rate limit denial after threshold</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>blocked_next=True</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1279,7 +1352,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Flow 02</t>
+          <t>Sensitive rate limit.</t>
         </is>
       </c>
     </row>
@@ -1404,14 +1477,29 @@
           <t>Session unlock for next command</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Voice engine initialized</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Wakeword pipeline object available (manual mic e2e pending).</t>
         </is>
       </c>
     </row>
@@ -1446,10 +1534,14 @@
           <t>Authentication succeeds only with valid PIN</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Authenticated as owner.</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1469,7 +1561,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Flow 02</t>
+          <t>Low confidence fallback to PIN.</t>
         </is>
       </c>
     </row>
@@ -1594,14 +1686,29 @@
           <t>find_draft action generated</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>{"original_text":"tim file o d","actions":[{"intent":"find_draft","args":{"drive":"D:\\"},"risk":"low","reason":"User asked to find draft/file in D drive"}],"needs_confirmation":false}</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Basic router.</t>
         </is>
       </c>
     </row>
@@ -1636,9 +1743,14 @@
           <t>Each sub-action evaluated by policy</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>find_draft,send_zalo,send_bulk_email</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1658,7 +1770,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Flow 01 core behavior</t>
+          <t>Composite policy flatten.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add streamlit UI shell and shared execution engine
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -687,6 +687,130 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>Flow 02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UI shell exists</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Repo has Flow 04 code</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>futureos/ui_app.py</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>File exists and importable</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ui_exists=True</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>UI shell file exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UI dependency</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pip install requirements</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>import streamlit</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Import success</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>streamlit import ok</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>UI dependency available.</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1389,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Actor is locked until 2026-03-21T16:52:03.993437+00:00.</t>
+          <t>Actor is locked until 2026-03-21T16:58:59.110423+00:00.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>

<commit_message>
feat: add durable queue and background worker runtime
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -557,7 +557,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -805,12 +805,136 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>UI dependency available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Queue process once</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Active session + queued command</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>worker run_once</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Task done and removed from queue</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{"ok": true, "task_id": "faa702c4-64f4-4c04-a0a6-d5b48125875c", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "User asked to find draft/file in D drive"}], "needs_confirmation": false}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Queue enqueue/process one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dead letter fallback</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Queued task with missing session</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>worker run_once</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Task moved to dead letter after retries</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>{"ok": false, "task_id": "dc373bfa-faab-4287-8134-1e42a4d12ca1", "error": "Session missing/expired for queued task."}</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Dead-letter on unrecoverable task.</t>
         </is>
       </c>
     </row>
@@ -952,7 +1076,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1014,7 +1138,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1076,7 +1200,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1138,7 +1262,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1285,7 +1409,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1347,7 +1471,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1389,7 +1513,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Actor is locked until 2026-03-21T16:58:59.110423+00:00.</t>
+          <t>Actor is locked until 2026-03-21T17:17:20.259264+00:00.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1409,7 +1533,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1471,7 +1595,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1618,7 +1742,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1680,7 +1804,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1827,7 +1951,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1889,7 +2013,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">

</xml_diff>

<commit_message>
feat: hardening sprint 1 reliability and security controls
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -847,7 +847,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>{"ok": true, "task_id": "faa702c4-64f4-4c04-a0a6-d5b48125875c", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "User asked to find draft/file in D drive"}], "needs_confirmation": false}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
+          <t>{"ok": true, "task_id": "dfda799e-551f-445f-beaf-e3f8c62bfcd2", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "User asked to find draft/file in D drive"}], "needs_confirmation": false}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>{"ok": false, "task_id": "dc373bfa-faab-4287-8134-1e42a4d12ca1", "error": "Session missing/expired for queued task."}</t>
+          <t>{"ok": false, "task_id": "89a967c5-837f-4837-826a-2d6064cf4dcd", "error": "Session missing/expired for queued task."}</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -935,6 +935,130 @@
       <c r="L8" t="inlineStr">
         <is>
           <t>Dead-letter on unrecoverable task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Queue idempotency</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Same idempotency key</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>enqueue same key twice</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Only one queued task remains</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>a=4a67ad65-4f5a-4529-9b7b-01290a14e9fe,b=4a67ad65-4f5a-4529-9b7b-01290a14e9fe,queued=1</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Idempotency blocks duplicate queue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Queue cancel</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Queued task exists</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>cancel-task &lt;id&gt;</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Task marked cancelled and not processed</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>cancel_ok=True</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Queued task cancel supported.</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1575,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>audit_exists=True</t>
+          <t>audit_exists=True,chain_ok=True</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1476,7 +1600,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Audit log exists.</t>
+          <t>Audit log exists and integrity chain verifies.</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1637,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Actor is locked until 2026-03-21T17:17:20.259264+00:00.</t>
+          <t>Actor is locked until 2026-03-21T17:31:48.001412+00:00.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>

<commit_message>
feat: add core file operations and vietnamese create-move parsing
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -847,7 +847,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>{"ok": true, "task_id": "dfda799e-551f-445f-beaf-e3f8c62bfcd2", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "User asked to find draft/file in D drive"}], "needs_confirmation": false}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
+          <t>{"ok": true, "task_id": "77b4752b-37ee-47c0-8290-a9eec44c3e8d", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "User asked to find draft/file in D drive"}], "needs_confirmation": false}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>{"ok": false, "task_id": "89a967c5-837f-4837-826a-2d6064cf4dcd", "error": "Session missing/expired for queued task."}</t>
+          <t>{"ok": false, "task_id": "d1dba0a9-19c5-4f94-8728-219cab67c758", "error": "Session missing/expired for queued task."}</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>a=4a67ad65-4f5a-4529-9b7b-01290a14e9fe,b=4a67ad65-4f5a-4529-9b7b-01290a14e9fe,queued=1</t>
+          <t>a=60dce63a-1bcc-464d-9605-beb69bffaaf3,b=60dce63a-1bcc-464d-9605-beb69bffaaf3,queued=1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1059,6 +1059,68 @@
       <c r="L10" t="inlineStr">
         <is>
           <t>Queued task cancel supported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>F-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>VN command create+move</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>VN command input</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tao thu muc zzz...di chuyen...</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Plan includes dir_create and path_move</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>dir_create,path_move</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>VN create+move command parsing.</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1699,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Actor is locked until 2026-03-21T17:31:48.001412+00:00.</t>
+          <t>Actor is locked until 2026-03-21T17:44:00.925565+00:00.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>

<commit_message>
feat: hybrid nlu v2 with vietnamese normalization and broad fileops tests
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -542,7 +542,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>steps=3</t>
+          <t>steps=2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>{"ok": true, "task_id": "77b4752b-37ee-47c0-8290-a9eec44c3e8d", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "User asked to find draft/file in D drive"}], "needs_confirmation": false}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
+          <t>{"ok": true, "task_id": "b25e8e98-0621-4a79-b5c9-5adf55892da8", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "Find draft in D drive"}], "needs_confirmation": false, "confidence": 0.72, "ambiguities": []}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>{"ok": false, "task_id": "d1dba0a9-19c5-4f94-8728-219cab67c758", "error": "Session missing/expired for queued task."}</t>
+          <t>{"ok": false, "task_id": "1bb999af-530e-4000-8fcc-7ecf38827228", "error": "Session missing/expired for queued task."}</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>a=60dce63a-1bcc-464d-9605-beb69bffaaf3,b=60dce63a-1bcc-464d-9605-beb69bffaaf3,queued=1</t>
+          <t>a=2832deb4-8091-40ef-a4a4-8338e0a7939b,b=2832deb4-8091-40ef-a4a4-8338e0a7939b,queued=1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1121,6 +1121,316 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>VN create+move command parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>VN move parsing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>VN command</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>di chuyen thu muc zzz vao backup o d</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Plan includes path_move</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>path_move</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>VN move parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>F-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>VN copy parsing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>VN command</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>sao chep thu muc zzz vao backup o d</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Plan includes path_copy</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>path_copy</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>VN copy parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>VN rename parsing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>VN command</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>doi ten thu muc zzz thanh zzz_new</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Plan includes path_rename</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>path_rename</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>VN rename parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>VN zip parsing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>VN command</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nen thu muc zzz vao backup o d</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Plan includes path_zip</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>path_zip</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>VN zip parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>F-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VN abbrev+typo parsing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>VN shorthand/typo command</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>tao tm zzz o desktp roi dc vao backup o d</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Plan includes dir_create and path_move</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>dir_create,path_move</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Abbrev+typo VN parsing.</t>
         </is>
       </c>
     </row>
@@ -1699,7 +2009,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Actor is locked until 2026-03-21T17:44:00.925565+00:00.</t>
+          <t>Actor is locked until 2026-03-22T02:12:06.667483+00:00.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2122,7 +2432,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>{"original_text":"tim file o d","actions":[{"intent":"find_draft","args":{"drive":"D:\\"},"risk":"low","reason":"User asked to find draft/file in D drive"}],"needs_confirmation":false}</t>
+          <t>{"original_text":"tim file o d","actions":[{"intent":"find_draft","args":{"drive":"D:\\"},"risk":"low","reason":"Find draft in D drive"}],"needs_confirmation":false,"confidence":0.72,"ambiguities":[]}</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2179,7 +2489,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>find_draft,send_zalo,send_bulk_email</t>
+          <t>send_zalo,send_bulk_email</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">

</xml_diff>

<commit_message>
hardening: improve vn fileops reliability and cli entrypoint
</commit_message>
<xml_diff>
--- a/TEST_CASES.xlsx
+++ b/TEST_CASES.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -847,7 +847,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>{"ok": true, "task_id": "b25e8e98-0621-4a79-b5c9-5adf55892da8", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "Find draft in D drive"}], "needs_confirmation": false, "confidence": 0.72, "ambiguities": []}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
+          <t>{"ok": true, "task_id": "68894213-ce32-4ced-a656-c73e2a497978", "result": {"ok": true, "plan": {"original_text": "tim file o d", "actions": [{"intent": "find_draft", "args": {"drive": "D:\\"}, "risk": "low", "reason": "Find draft in D drive"}], "needs_confirmation": false, "confidence": 0.72, "ambiguities": []}, "policy": [{"intent": "find_draft", "allowed": true, "reason": "Allowed by role policy.", "needs_confirmation": false}], "results": [{"ok": true, "action": "find_draft", "detail": "Found 5 candidate file(s)", "payload": {"files": ["D:\\Study\\For C++\\1.txt", "D:\\Study\\For C++\\2.txt", "D:\\Study\\For C++\\3.txt", "D:\\Study\\For C++\\4.txt", "D:\\Study\\For C++\\5.txt"]}}]}}</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>{"ok": false, "task_id": "1bb999af-530e-4000-8fcc-7ecf38827228", "error": "Session missing/expired for queued task."}</t>
+          <t>{"ok": false, "task_id": "a5df0c4f-49f3-4e82-98d5-f763f76f0e82", "error": "Session missing/expired for queued task."}</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>a=2832deb4-8091-40ef-a4a4-8338e0a7939b,b=2832deb4-8091-40ef-a4a4-8338e0a7939b,queued=1</t>
+          <t>a=d15ca91f-aeb1-4c77-ac1a-fd110cdf2d9b,b=d15ca91f-aeb1-4c77-ac1a-fd110cdf2d9b,queued=1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1431,6 +1431,68 @@
       <c r="L16" t="inlineStr">
         <is>
           <t>Abbrev+typo VN parsing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>F-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Original VN sentence parsing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Complex VN typo/abbrev sentence</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>tim file d? liueeju...</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Plan includes file_search+dir_create+path_move</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>file_search,dir_create,path_move</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>codex</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Original complex VN sentence parsing.</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2071,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Actor is locked until 2026-03-22T02:12:06.667483+00:00.</t>
+          <t>Actor is locked until 2026-03-22T02:36:01.040639+00:00.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>